<commit_message>
release(kg): publish validated asserted-only v3.0.0 and align data paper
</commit_message>
<xml_diff>
--- a/metadata/samples/EB_Sample_Map_FourthTrip2.xlsx
+++ b/metadata/samples/EB_Sample_Map_FourthTrip2.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abdelhm/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5DE2FC-2EB8-9A40-9B83-E0D57911E3DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3739581B-D102-7048-BF2A-70D1C13F02C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="44800" windowHeight="23040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18200" yWindow="2420" windowWidth="26120" windowHeight="18340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EB-Sample Map (Trip 4)" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0" calcOnSave="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Extraction Blank</t>
   </si>
@@ -43,12 +43,6 @@
     <t>EB2</t>
   </si>
   <si>
-    <t>3, 7, 19, 21, 32, 39, 48, 31 (PRr1/Sr1 only)</t>
-  </si>
-  <si>
-    <t>S3PRr1, S3Sr1, S3Dr1, S7PRr1, S7Sr1, S7Dr1, S19PRr1, S19Sr1, S19Dr1, S21PRr1, S21Sr1, S21Dr1, S32PRr1, S32Sr1, S32Dr1, S39PRr1, S39Sr1, S39Dr1, S48PRr1, S48Sr1, S48Dr1, S31PRr1, S31Sr1</t>
-  </si>
-  <si>
     <t>EB3</t>
   </si>
   <si>
@@ -64,9 +58,6 @@
     <t>5, 6, 10, 20, 24, 34, 40, 52, 1 (PRr1/Sr1 only)</t>
   </si>
   <si>
-    <t>S5PRr1, S5Sr1, S5Dr1, S6PRr1, S6Sr1, S6Dr1, S10PRr1, S10Sr1, S10Dr1, S20PRr1, S20Sr1, S20Dr1, S24PRr1, S24Sr1, S24Dr1, S34PRr1, S34Sr1, S34Dr1, S40PRr1, S40Sr1, S40Dr1, S52PRr1, S52Sr1, S52Dr1, S1PRr1, S1Sr1</t>
-  </si>
-  <si>
     <t>EB5</t>
   </si>
   <si>
@@ -76,18 +67,9 @@
     <t>S19PRr1, S19Sr1, S19Dr1, S26PRr1, S26Sr1, S26Dr1, S42PRr1, S42Sr1, S42Dr1</t>
   </si>
   <si>
-    <t>EB</t>
-  </si>
-  <si>
     <t>4,8,11,36,59</t>
   </si>
   <si>
-    <t>S4PRr1, S4Sr1, S4Dr1, S8PRr1, S8Sr1, S8Dr1, S11PRr1, S11Sr1, S11Dr1, S36PRr1, S36Sr1, S36Dr1, S59PRr1, S59Sr1, S59Dr1</t>
-  </si>
-  <si>
-    <t>The EB for three days extraction wasn't sequenced  sites 22,28,35,43,53,46,13,25,54,55,44,38,41,33,2,27,51,16,59,57,56,49,45</t>
-  </si>
-  <si>
     <t>EB Index</t>
   </si>
   <si>
@@ -116,6 +98,27 @@
   </si>
   <si>
     <t># Sequenced</t>
+  </si>
+  <si>
+    <t>S4PRr1, S4Sr1, S4Dr1, S8PRr1, S8Sr1, S8Dr1, S11PRr1, S11Sr1, S11Dr1, S36PRr1, S36Sr1, S36Dr1,  S59Sr1</t>
+  </si>
+  <si>
+    <t>S3PRr1, S3Sr1, S3Dr1, S7PRr1, S7Sr1, S7Dr1, S14PRr1, S14Sr1, S14Dr1, S21PRr1, S21Sr1, S21Dr1, S32PRr1, S32Sr1, S32Dr1, S39PRr1, S39Sr1, S39Dr1, S48PRr1, S48Sr1, S48Dr1, S31PRr1, S31Sr1</t>
+  </si>
+  <si>
+    <t>S5PRr1, S5Sr1, S5Dr1, S10PRr1, S10Sr1, S10Dr1, S20PRr1, S20Sr1, S20Dr1, S24PRr1, S24Sr1, S24Dr1, S34PRr1, S34Sr1, S34Dr1, S40PRr1, S40Sr1, S40Dr1, S52PRr1, S52Sr1, S52Dr1, S1PRr1, S1Sr1</t>
+  </si>
+  <si>
+    <t>3, 7, 14, 21, 32, 39, 48, 31 (PRr1/Sr1 only)</t>
+  </si>
+  <si>
+    <t>SEB</t>
+  </si>
+  <si>
+    <t>The PCR blank was not sequenced in this run, as the index assigned to it was shared with another sample from a different trip, and it was therefore excluded in favour of retaining the actual sample."</t>
+  </si>
+  <si>
+    <t>The EB for three days extraction wasn't sequenced  sites 2, 13, 16, 18, 22, 25, 27, 28, 33, 35, 37, 38, 41, 43, 44, 45, 46, 47, 49, 51, 53, 54, 55, 56, 57, 58, 59(PRr1, 59Dr1), 60</t>
   </si>
 </sst>
 </file>
@@ -251,14 +254,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -575,10 +578,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>31</v>
+        <v>16</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>25</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
@@ -589,19 +592,19 @@
     </row>
     <row r="2" spans="1:5" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C2" s="7">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
@@ -609,7 +612,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C3" s="7">
         <v>22</v>
@@ -626,85 +629,91 @@
         <v>6</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C4" s="7">
         <v>23</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C5" s="7">
         <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C6" s="7">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C7" s="7">
         <v>9</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
-        <v>29</v>
+      <c r="A8" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>30</v>
+        <v>24</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
+      <c r="A9" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>